<commit_message>
Log every prompt sent for a check run, and require mismatches be surfaced plainly
Each run now writes one log file per case+datetime under
C:\logs\apipromptevaluator, capturing every check's system prompt, user
prompt and raw LLM response so a run is fully auditable after the fact.
The assessor's system prompt also now explicitly requires any identified
mismatch to be reported without softening or masking it.

Also updates CHK-001's query plan to match the QA checks CSV: adds
Existing Plans & Portfolios (E), protection plan and fund holdings
queries, an emergency-fund consistency group, and the check's new
out-of-scope boundary.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/QA-Checks/Assessment Checks & Prompts QA CA v1.0-n.xlsx
+++ b/docs/QA-Checks/Assessment Checks & Prompts QA CA v1.0-n.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\work\Prompt-Evaluator-Forms\docs\QA-Checks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{474BE9F4-F31A-44E6-810D-3A1074194A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED1F099-11AB-457A-8B56-B0D530BE6FD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{CFAFE921-0325-496C-8F99-317BA935E5B4}"/>
+    <workbookView xWindow="-28920" yWindow="4785" windowWidth="29040" windowHeight="15720" xr2:uid="{CFAFE921-0325-496C-8F99-317BA935E5B4}"/>
   </bookViews>
   <sheets>
     <sheet name="Assessment Checks v1.0" sheetId="3" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="187">
   <si>
     <t>Check ID</t>
   </si>
@@ -82,12 +82,6 @@
   </si>
   <si>
     <t>Not required for this check</t>
-  </si>
-  <si>
-    <t>Client Authority (A)
-Know Your Client (B)
-Meeting &amp; Communications (C)
-Recommendations &amp; Advice (I)</t>
   </si>
   <si>
     <t>Where client information/facts have been included in the Suitability Report they are consistent with the evidence provided?</t>
@@ -1406,13 +1400,6 @@
     <t>Application; acceptance; cancellation; implementation evidence; client confirmation; post-sale correspondence; review/service records</t>
   </si>
   <si>
-    <t xml:space="preserve">Look for data mismatches and unsupported figures. 
-- Essential facts (personal details, tax status, employment etc.)
-- Financial situation (income/expenditure, assets/liabilities &amp; state pension entitlement)
-- Existing products (pensions and investments)
-</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Are the details of the recommendations and goals consistent with the evidence provided?
 </t>
@@ -1505,6 +1492,30 @@
       <t xml:space="preserve">
 </t>
     </r>
+  </si>
+  <si>
+    <t>Personal details (name, age, date of birth, marital status, dependants, employment, residency, tax status etc.).
+Financial situation (income, expenditure, assets, liabilities, emergency funds, state pension entitlement).
+Existing products (investments, pensions, protection plans and provider details).
+Data mismatches, unsupported statements, missing evidence and conflicting information across documents.
+Values, dates, names and holdings should reconcile across the file.
+Do not assess:
+Suitability of recommendations.
+Attitude to Risk.
+Capacity for Loss.
+Knowledge and experience.
+Investment suitability.
+Product selection rationale.</t>
+  </si>
+  <si>
+    <t>Where client and family information and factual circumstances have been included in the Suitability Report, they are consistent with the supporting client file evidence.</t>
+  </si>
+  <si>
+    <t>Client Authority (A)
+Know Your Client (B)
+Meeting &amp; Communications (C)
+Existing Plans &amp; Portfolios (E)
+Recommendations &amp; Advice (I)</t>
   </si>
 </sst>
 </file>
@@ -2319,250 +2330,250 @@
         <v>11</v>
       </c>
       <c r="E2" s="34" t="s">
-        <v>12</v>
+        <v>186</v>
       </c>
       <c r="F2" s="34" t="s">
+        <v>185</v>
+      </c>
+      <c r="G2" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="H2" s="34" t="s">
         <v>13</v>
-      </c>
-      <c r="G2" s="40" t="s">
-        <v>179</v>
-      </c>
-      <c r="H2" s="34" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="306" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>16</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F3" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="G3" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="G3" s="38" t="s">
-        <v>19</v>
-      </c>
       <c r="H3" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="276" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="E4" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="G4" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="39" t="s">
-        <v>181</v>
-      </c>
-      <c r="G4" s="39" t="s">
+      <c r="H4" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="H4" s="8" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="303.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>28</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="G5" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>182</v>
-      </c>
-      <c r="G5" s="38" t="s">
+      <c r="H5" s="9" t="s">
         <v>31</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="315" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="D6" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="36" t="s">
+      <c r="F6" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="H6" s="8" t="s">
         <v>38</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="215.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="E7" s="22" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="F7" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F7" s="9" t="s">
+      <c r="G7" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="G7" s="38" t="s">
+      <c r="H7" s="9" t="s">
         <v>46</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="265.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="G8" s="39" t="s">
         <v>51</v>
       </c>
-      <c r="F8" s="22" t="s">
-        <v>183</v>
-      </c>
-      <c r="G8" s="39" t="s">
-        <v>52</v>
-      </c>
       <c r="H8" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="189.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>53</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>54</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>10</v>
       </c>
       <c r="D9" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="36" t="s">
+      <c r="G9" s="38" t="s">
         <v>56</v>
       </c>
-      <c r="G9" s="38" t="s">
+      <c r="H9" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="291" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="E10" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="F10" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="G10" s="39" t="s">
         <v>63</v>
       </c>
-      <c r="F10" s="23" t="s">
-        <v>184</v>
-      </c>
-      <c r="G10" s="39" t="s">
+      <c r="H10" s="8" t="s">
         <v>64</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="306.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="C11" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="D11" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="E11" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="F11" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="F11" s="22" t="s">
-        <v>71</v>
-      </c>
       <c r="G11" s="41" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -2585,112 +2596,112 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="C1" s="20" t="s">
         <v>73</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="C2" s="20" t="s">
         <v>76</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B3" s="29" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="C3" s="30" t="s">
         <v>79</v>
-      </c>
-      <c r="C3" s="30" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B4" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="C4" s="20" t="s">
         <v>82</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="19" t="s">
         <v>84</v>
       </c>
-      <c r="B5" s="19" t="s">
+      <c r="C5" s="20" t="s">
         <v>85</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="C6" s="20" t="s">
         <v>88</v>
-      </c>
-      <c r="C6" s="20" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="51.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="19" t="s">
+      <c r="C7" s="37" t="s">
         <v>91</v>
-      </c>
-      <c r="C7" s="37" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="51" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>93</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="C8" s="37" t="s">
         <v>94</v>
-      </c>
-      <c r="C8" s="37" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B9" s="19" t="s">
+      <c r="C9" s="20" t="s">
         <v>97</v>
-      </c>
-      <c r="C9" s="20" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="B10" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="B10" s="19" t="s">
+      <c r="C10" s="20" t="s">
         <v>100</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2727,7 +2738,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="18" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>2</v>
@@ -2739,7 +2750,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>5</v>
@@ -2748,51 +2759,51 @@
         <v>6</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="2" spans="1:12" s="28" customFormat="1" ht="182" x14ac:dyDescent="0.35">
       <c r="A2" s="26" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="27" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="C2" s="27" t="s">
         <v>107</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>108</v>
       </c>
       <c r="D2" s="27" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="27" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="27" t="s">
         <v>109</v>
       </c>
-      <c r="F2" s="27" t="s">
+      <c r="G2" s="27" t="s">
         <v>110</v>
       </c>
-      <c r="G2" s="27" t="s">
+      <c r="H2" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="H2" s="27" t="s">
+      <c r="I2" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="I2" s="27" t="s">
+      <c r="J2" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="L2" s="27" t="s">
         <v>114</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>32</v>
-      </c>
-      <c r="L2" s="27" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:12" s="16" customFormat="1" ht="91" x14ac:dyDescent="0.35">
@@ -2810,365 +2821,365 @@
         <v>11</v>
       </c>
       <c r="F3" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="G3" s="27" t="s">
         <v>116</v>
       </c>
-      <c r="G3" s="27" t="s">
+      <c r="H3" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="15" t="s">
         <v>117</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="J3" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="K3" s="15" t="s">
         <v>13</v>
-      </c>
-      <c r="I3" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="J3" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="K3" s="15" t="s">
-        <v>14</v>
       </c>
       <c r="L3" s="15"/>
     </row>
     <row r="4" spans="1:12" ht="208" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>16</v>
-      </c>
       <c r="C4" s="17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F4" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="G4" s="31" t="s">
         <v>120</v>
       </c>
-      <c r="G4" s="31" t="s">
+      <c r="H4" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="I4" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="J4" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J4" s="6" t="s">
-        <v>124</v>
-      </c>
       <c r="K4" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="364" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="E5" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="8" t="s">
+      <c r="G5" s="27" t="s">
         <v>126</v>
       </c>
-      <c r="G5" s="27" t="s">
+      <c r="H5" s="8" t="s">
         <v>127</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="I5" s="4" t="s">
         <v>128</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>130</v>
-      </c>
       <c r="K5" s="8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="306.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>28</v>
-      </c>
       <c r="C6" s="17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F6" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="G6" s="31" t="s">
         <v>131</v>
       </c>
-      <c r="G6" s="31" t="s">
+      <c r="H6" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="I6" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="J6" s="6" t="s">
-        <v>135</v>
-      </c>
       <c r="K6" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="143" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="C7" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="E7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="20" t="s">
         <v>136</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="20" t="s">
+      <c r="G7" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="G7" s="27" t="s">
+      <c r="H7" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="I7" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="H7" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7" s="4" t="s">
+      <c r="J7" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>140</v>
-      </c>
       <c r="K7" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="312" x14ac:dyDescent="0.35">
       <c r="A8" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="17" t="s">
+        <v>140</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="E8" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="20" t="s">
         <v>141</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" s="20" t="s">
+      <c r="G8" s="31" t="s">
         <v>142</v>
       </c>
-      <c r="G8" s="31" t="s">
+      <c r="H8" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="H8" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="I8" s="6" t="s">
+      <c r="J8" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="J8" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="K8" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L8" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="408.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="C9" s="12" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F9" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="G9" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="H9" s="22" t="s">
         <v>148</v>
       </c>
-      <c r="H9" s="22" t="s">
+      <c r="I9" s="4" t="s">
         <v>149</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="J9" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>151</v>
-      </c>
       <c r="K9" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="273" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="C10" s="17" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="22" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="G10" s="31" t="s">
+        <v>152</v>
+      </c>
+      <c r="H10" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="G10" s="31" t="s">
+      <c r="I10" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="H10" s="22" t="s">
-        <v>56</v>
-      </c>
-      <c r="I10" s="6" t="s">
+      <c r="J10" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="J10" s="6" t="s">
-        <v>155</v>
-      </c>
       <c r="K10" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L10" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="390" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="C11" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="E11" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" s="8" t="s">
+      <c r="G11" s="27" t="s">
         <v>157</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="H11" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="H11" s="20" t="s">
+      <c r="I11" s="4" t="s">
         <v>159</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="J11" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>161</v>
-      </c>
       <c r="K11" s="8" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="273" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="E12" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="9" t="s">
+      <c r="G12" s="31" t="s">
         <v>163</v>
       </c>
-      <c r="G12" s="31" t="s">
+      <c r="H12" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="H12" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="I12" s="6" t="s">
+      <c r="J12" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="J12" s="6" t="s">
-        <v>166</v>
-      </c>
       <c r="K12" s="9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
   </sheetData>
@@ -3197,112 +3208,112 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="C1" s="20" t="s">
         <v>73</v>
-      </c>
-      <c r="C1" s="20" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A2" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" s="20" t="s">
         <v>167</v>
-      </c>
-      <c r="B2" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C2" s="20" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="29" t="s">
+        <v>168</v>
+      </c>
+      <c r="B3" s="29" t="s">
         <v>169</v>
       </c>
-      <c r="B3" s="29" t="s">
-        <v>170</v>
-      </c>
       <c r="C3" s="30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A4" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B5" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>85</v>
-      </c>
-      <c r="C5" s="20" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A6" s="19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A7" s="19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B7" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="C7" s="20" t="s">
         <v>173</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A8" s="19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C8" s="20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="19" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="29" x14ac:dyDescent="0.35">
       <c r="A10" s="24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B10" s="24" t="s">
+        <v>176</v>
+      </c>
+      <c r="C10" s="25" t="s">
         <v>177</v>
-      </c>
-      <c r="C10" s="25" t="s">
-        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>